<commit_message>
[Vikas]Updated Transactions And it's IO files along with OptimizedJsonExcelComparator class
</commit_message>
<xml_diff>
--- a/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
+++ b/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\wings-testautomation\src\main\resources\menuItems\Sales\Transactions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\Wings-Automation\src\main\resources\menuItems\Sales\Transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03D237D6-D215-4327-9226-4F46A08763AF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3825DB9A-5FF2-431D-ABDB-ADE13D4B3632}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="938" activeTab="2"/>
+    <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="938" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="616">
   <si>
     <t>TableNames</t>
   </si>
@@ -1887,12 +1887,15 @@
   </si>
   <si>
     <t>Cost Of Goods Sold per Unit</t>
+  </si>
+  <si>
+    <t>ī</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1901,7 +1904,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1920,6 +1923,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1933,12 +1942,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2246,7 +2259,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2516,7 +2529,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2578,7 +2591,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2636,7 +2649,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2835,7 +2848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3205,7 +3218,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3479,7 +3492,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3735,7 +3748,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3769,7 +3782,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3803,7 +3816,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3868,7 +3881,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3988,7 +4001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -4162,7 +4175,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -4607,7 +4620,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -4711,7 +4724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -4815,7 +4828,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -4900,11 +4913,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:BX18"/>
+  <dimension ref="A1:BX28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
@@ -5905,23 +5918,23 @@
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="E5" t="s">
-        <v>138</v>
+      <c r="E5">
+        <v>8967</v>
       </c>
       <c r="F5" t="s">
         <v>139</v>
       </c>
-      <c r="G5" t="s">
-        <v>53</v>
-      </c>
-      <c r="H5" t="s">
-        <v>53</v>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
       </c>
       <c r="I5" t="s">
         <v>193</v>
       </c>
       <c r="J5" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="K5" t="s">
         <v>195</v>
@@ -5939,58 +5952,58 @@
         <v>143</v>
       </c>
       <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
         <v>1</v>
       </c>
-      <c r="Q5">
+      <c r="U5">
         <v>1</v>
       </c>
-      <c r="R5">
+      <c r="V5">
         <v>1</v>
       </c>
-      <c r="S5">
+      <c r="W5">
         <v>1</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
       </c>
       <c r="X5">
         <v>500.14</v>
       </c>
       <c r="Y5">
-        <v>500.14</v>
+        <v>0</v>
       </c>
       <c r="Z5">
         <v>250.14</v>
       </c>
       <c r="AA5">
-        <v>250.14</v>
-      </c>
-      <c r="AB5" s="4">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="4">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="5">
         <v>0</v>
       </c>
       <c r="AD5">
         <v>1.1100000000000001</v>
       </c>
       <c r="AE5">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="AF5">
-        <v>1.1499999999999999</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="AG5">
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="s">
         <v>196</v>
@@ -5999,7 +6012,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ5">
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="s">
         <v>196</v>
@@ -6008,7 +6021,7 @@
         <v>1.21</v>
       </c>
       <c r="AM5">
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AN5" t="s">
         <v>197</v>
@@ -6017,10 +6030,10 @@
         <v>1.26</v>
       </c>
       <c r="AP5">
-        <v>3.12</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>57</v>
+        <v>0</v>
+      </c>
+      <c r="AQ5">
+        <v>0</v>
       </c>
       <c r="AR5" t="s">
         <v>145</v>
@@ -6032,31 +6045,31 @@
         <v>147</v>
       </c>
       <c r="AU5">
-        <v>239.1</v>
+        <v>0</v>
       </c>
       <c r="AV5">
         <v>12</v>
       </c>
       <c r="AW5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AX5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AY5">
         <v>0</v>
       </c>
       <c r="AZ5">
-        <v>2.39</v>
+        <v>0</v>
       </c>
       <c r="BA5">
-        <v>31.09</v>
+        <v>0</v>
       </c>
       <c r="BB5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BC5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BD5" t="s">
         <v>198</v>
@@ -6071,55 +6084,55 @@
         <v>201</v>
       </c>
       <c r="BH5" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="BI5" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="BJ5" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="BK5" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="BL5" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="BM5" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="BN5">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="BO5">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="BP5">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="BQ5">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="BR5">
-        <v>1.58</v>
+        <v>1.59</v>
       </c>
       <c r="BS5" s="1">
-        <v>45859</v>
+        <v>45862</v>
       </c>
       <c r="BT5" s="1">
-        <v>45860</v>
+        <v>45863</v>
       </c>
       <c r="BU5" s="1">
-        <v>45861</v>
-      </c>
-      <c r="BV5" t="s">
-        <v>53</v>
-      </c>
-      <c r="BW5" t="s">
-        <v>53</v>
-      </c>
-      <c r="BX5" t="s">
-        <v>53</v>
+        <v>45864</v>
+      </c>
+      <c r="BV5" s="6">
+        <v>1</v>
+      </c>
+      <c r="BW5" s="6">
+        <v>1</v>
+      </c>
+      <c r="BX5" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:76" x14ac:dyDescent="0.25">
@@ -6135,23 +6148,23 @@
       <c r="D6" t="s">
         <v>191</v>
       </c>
-      <c r="E6" t="s">
-        <v>138</v>
+      <c r="E6">
+        <v>8967</v>
       </c>
       <c r="F6" t="s">
         <v>139</v>
       </c>
-      <c r="G6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H6" t="s">
-        <v>53</v>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
       </c>
       <c r="I6" t="s">
         <v>193</v>
       </c>
       <c r="J6" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="K6" t="s">
         <v>195</v>
@@ -6169,58 +6182,58 @@
         <v>143</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <v>500.14</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <v>500.14</v>
       </c>
       <c r="Z6">
         <v>250.14</v>
       </c>
       <c r="AA6">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="4">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="4">
+        <v>250.14</v>
+      </c>
+      <c r="AB6" s="5">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="5">
         <v>0</v>
       </c>
       <c r="AD6">
         <v>1.1100000000000001</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <v>2.78</v>
       </c>
       <c r="AF6">
-        <v>1.1599999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <v>2.88</v>
       </c>
       <c r="AH6" t="s">
         <v>196</v>
@@ -6229,7 +6242,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AK6" t="s">
         <v>196</v>
@@ -6238,7 +6251,7 @@
         <v>1.21</v>
       </c>
       <c r="AM6">
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AN6" t="s">
         <v>197</v>
@@ -6247,10 +6260,10 @@
         <v>1.26</v>
       </c>
       <c r="AP6">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="s">
-        <v>57</v>
+        <v>3.12</v>
+      </c>
+      <c r="AQ6">
+        <v>0</v>
       </c>
       <c r="AR6" t="s">
         <v>145</v>
@@ -6262,31 +6275,31 @@
         <v>147</v>
       </c>
       <c r="AU6">
-        <v>0</v>
+        <v>239.1</v>
       </c>
       <c r="AV6">
         <v>12</v>
       </c>
       <c r="AW6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AX6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AY6">
         <v>0</v>
       </c>
       <c r="AZ6">
-        <v>0</v>
+        <v>2.39</v>
       </c>
       <c r="BA6">
-        <v>0</v>
+        <v>31.09</v>
       </c>
       <c r="BB6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BC6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BD6" t="s">
         <v>198</v>
@@ -6301,55 +6314,55 @@
         <v>201</v>
       </c>
       <c r="BH6" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="BI6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="BJ6" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="BK6" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="BL6" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="BM6" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="BN6">
-        <v>1.33</v>
+        <v>1.32</v>
       </c>
       <c r="BO6">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
       <c r="BP6">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="BQ6">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="BR6">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
       <c r="BS6" s="1">
-        <v>45862</v>
+        <v>45859</v>
       </c>
       <c r="BT6" s="1">
-        <v>45863</v>
+        <v>45860</v>
       </c>
       <c r="BU6" s="1">
-        <v>45864</v>
-      </c>
-      <c r="BV6" t="s">
-        <v>53</v>
-      </c>
-      <c r="BW6" t="s">
-        <v>53</v>
-      </c>
-      <c r="BX6" t="s">
-        <v>53</v>
+        <v>45861</v>
+      </c>
+      <c r="BV6" s="6">
+        <v>1</v>
+      </c>
+      <c r="BW6" s="6">
+        <v>1</v>
+      </c>
+      <c r="BX6" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:76" x14ac:dyDescent="0.25">
@@ -6712,85 +6725,85 @@
     <row r="13" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="AA13" s="3">
         <f t="shared" si="0"/>
-        <v>250.14</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="3">
         <f t="shared" si="5"/>
-        <v>2.776554</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="3">
         <f t="shared" si="5"/>
-        <v>2.8766099999999999</v>
+        <v>0</v>
       </c>
       <c r="AJ13" s="3">
         <f>$R5*AI5</f>
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AM13" s="3">
         <f>$R5*AL5</f>
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AP13" s="3">
         <f>($AA13-AJ13-AM13)*AO5%</f>
-        <v>3.1232879999999996</v>
+        <v>0</v>
       </c>
       <c r="AS13" s="3">
         <f t="shared" si="1"/>
-        <v>11.036452000000001</v>
+        <v>0</v>
       </c>
       <c r="AU13" s="3">
         <f t="shared" si="2"/>
-        <v>239.10354799999999</v>
+        <v>0</v>
       </c>
       <c r="BA13" s="3">
         <f t="shared" si="3"/>
-        <v>31.08242576</v>
+        <v>0</v>
       </c>
       <c r="BB13" s="3">
         <f t="shared" si="4"/>
-        <v>270.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="AA14" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>250.14</v>
       </c>
       <c r="AE14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.776554</v>
       </c>
       <c r="AG14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.8766099999999999</v>
       </c>
       <c r="AJ14" s="3">
         <f>$R6*AI6</f>
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AM14" s="3">
         <f>$R6*AL6</f>
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AP14" s="3">
         <f>($AA14-AJ14-AM14)*AO6%</f>
-        <v>0</v>
+        <v>3.1232879999999996</v>
       </c>
       <c r="AS14" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>11.036452000000001</v>
       </c>
       <c r="AU14" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>239.10354799999999</v>
       </c>
       <c r="BA14" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31.08242576</v>
       </c>
       <c r="BB14" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>270.19</v>
       </c>
     </row>
     <row r="15" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -6836,7 +6849,7 @@
       </c>
     </row>
     <row r="16" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="27:54" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="27:72" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="AA17" s="3">
         <f>SUM(AA10:AA15)</f>
         <v>1205.0627899999999</v>
@@ -6878,7 +6891,7 @@
         <v>1349.27</v>
       </c>
     </row>
-    <row r="18" spans="27:54" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="27:72" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="AA18" s="3">
         <f>SUM(AA2:AA7)</f>
         <v>1205.06</v>
@@ -6934,6 +6947,11 @@
       <c r="BB18" s="3">
         <f t="shared" si="6"/>
         <v>1349.18</v>
+      </c>
+    </row>
+    <row r="28" spans="27:72" x14ac:dyDescent="0.25">
+      <c r="BT28" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>
@@ -6943,7 +6961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -7400,7 +7418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -7920,7 +7938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -8740,7 +8758,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -9560,7 +9578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -9670,7 +9688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>

</xml_diff>

<commit_message>
[Vikas]Updated Transactions In Purchase,Sales,Finance modules And it's IO files along with OptimizedJsonExcelComparator class
</commit_message>
<xml_diff>
--- a/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
+++ b/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\Wings-Automation\src\main\resources\menuItems\Sales\Transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3825DB9A-5FF2-431D-ABDB-ADE13D4B3632}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71E4B4F-0FF3-4C27-8033-DF2AE95BD35A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="938" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5918,7 +5918,7 @@
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="6">
         <v>8967</v>
       </c>
       <c r="F5" t="s">
@@ -6148,7 +6148,7 @@
       <c r="D6" t="s">
         <v>191</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="6">
         <v>8967</v>
       </c>
       <c r="F6" t="s">

</xml_diff>

<commit_message>
[Vikas]Updated transactions on Finance and Production modules along with their Excel files.Updated OptimizedJsonExcelComparator and APIClient utility  Code.
</commit_message>
<xml_diff>
--- a/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
+++ b/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\Wings-Automation\src\main\resources\menuItems\Sales\Transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77185577-FD6D-4B2D-A660-5EAA1B260204}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A13C3C1-4E32-441D-B3F6-2120CC5B5F85}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="938" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5950,7 +5950,7 @@
         <v>192</v>
       </c>
       <c r="J5" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="K5" t="s">
         <v>194</v>
@@ -5968,40 +5968,40 @@
         <v>142</v>
       </c>
       <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
         <v>1</v>
       </c>
-      <c r="Q5">
+      <c r="U5">
         <v>1</v>
       </c>
-      <c r="R5">
+      <c r="V5">
         <v>1</v>
       </c>
-      <c r="S5">
+      <c r="W5">
         <v>1</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
       </c>
       <c r="X5">
         <v>500.14</v>
       </c>
       <c r="Y5">
-        <v>500.14</v>
+        <v>0</v>
       </c>
       <c r="Z5">
         <v>250.14</v>
       </c>
       <c r="AA5">
-        <v>250.14</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="5">
         <v>0</v>
@@ -6013,13 +6013,13 @@
         <v>1.1100000000000001</v>
       </c>
       <c r="AE5">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="AF5">
-        <v>1.1499999999999999</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="AG5">
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="s">
         <v>195</v>
@@ -6028,7 +6028,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ5">
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="s">
         <v>195</v>
@@ -6037,7 +6037,7 @@
         <v>1.21</v>
       </c>
       <c r="AM5">
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AN5" t="s">
         <v>196</v>
@@ -6046,7 +6046,7 @@
         <v>1.26</v>
       </c>
       <c r="AP5">
-        <v>3.12</v>
+        <v>0</v>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -6061,31 +6061,31 @@
         <v>146</v>
       </c>
       <c r="AU5">
-        <v>239.1</v>
+        <v>0</v>
       </c>
       <c r="AV5">
         <v>12</v>
       </c>
       <c r="AW5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AX5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AY5">
         <v>0</v>
       </c>
       <c r="AZ5">
-        <v>2.39</v>
+        <v>0</v>
       </c>
       <c r="BA5">
-        <v>31.09</v>
+        <v>0</v>
       </c>
       <c r="BB5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BC5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BD5" t="s">
         <v>197</v>
@@ -6100,46 +6100,46 @@
         <v>200</v>
       </c>
       <c r="BH5" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="BI5" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="BJ5" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="BK5" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="BL5" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="BM5" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="BN5">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="BO5">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="BP5">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="BQ5">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="BR5">
-        <v>1.58</v>
+        <v>1.59</v>
       </c>
       <c r="BS5" s="1">
-        <v>45859</v>
+        <v>45862</v>
       </c>
       <c r="BT5" s="1">
-        <v>45860</v>
+        <v>45863</v>
       </c>
       <c r="BU5" s="1">
-        <v>45861</v>
+        <v>45864</v>
       </c>
       <c r="BV5" s="6">
         <v>1</v>
@@ -6180,7 +6180,7 @@
         <v>192</v>
       </c>
       <c r="J6" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="K6" t="s">
         <v>194</v>
@@ -6198,40 +6198,40 @@
         <v>142</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <v>500.14</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <v>500.14</v>
       </c>
       <c r="Z6">
         <v>250.14</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <v>250.14</v>
       </c>
       <c r="AB6" s="5">
         <v>0</v>
@@ -6243,13 +6243,13 @@
         <v>1.1100000000000001</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <v>2.78</v>
       </c>
       <c r="AF6">
-        <v>1.1599999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <v>2.88</v>
       </c>
       <c r="AH6" t="s">
         <v>195</v>
@@ -6258,7 +6258,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AK6" t="s">
         <v>195</v>
@@ -6267,7 +6267,7 @@
         <v>1.21</v>
       </c>
       <c r="AM6">
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AN6" t="s">
         <v>196</v>
@@ -6276,7 +6276,7 @@
         <v>1.26</v>
       </c>
       <c r="AP6">
-        <v>0</v>
+        <v>3.12</v>
       </c>
       <c r="AQ6">
         <v>0</v>
@@ -6291,31 +6291,31 @@
         <v>146</v>
       </c>
       <c r="AU6">
-        <v>0</v>
+        <v>239.1</v>
       </c>
       <c r="AV6">
         <v>12</v>
       </c>
       <c r="AW6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AX6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AY6">
         <v>0</v>
       </c>
       <c r="AZ6">
-        <v>0</v>
+        <v>2.39</v>
       </c>
       <c r="BA6">
-        <v>0</v>
+        <v>31.09</v>
       </c>
       <c r="BB6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BC6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BD6" t="s">
         <v>197</v>
@@ -6330,46 +6330,46 @@
         <v>200</v>
       </c>
       <c r="BH6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="BI6" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="BJ6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="BK6" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="BL6" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="BM6" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="BN6">
-        <v>1.33</v>
+        <v>1.32</v>
       </c>
       <c r="BO6">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
       <c r="BP6">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="BQ6">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="BR6">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
       <c r="BS6" s="1">
-        <v>45862</v>
+        <v>45859</v>
       </c>
       <c r="BT6" s="1">
-        <v>45863</v>
+        <v>45860</v>
       </c>
       <c r="BU6" s="1">
-        <v>45864</v>
+        <v>45861</v>
       </c>
       <c r="BV6" s="6">
         <v>1</v>
@@ -6747,86 +6747,86 @@
       <c r="D13" s="7"/>
       <c r="AA13" s="3">
         <f t="shared" si="0"/>
-        <v>250.14</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="3">
         <f t="shared" si="5"/>
-        <v>2.776554</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="3">
         <f t="shared" si="5"/>
-        <v>2.8766099999999999</v>
+        <v>0</v>
       </c>
       <c r="AJ13" s="3">
         <f>$R5*AI5</f>
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AM13" s="3">
         <f>$R5*AL5</f>
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AP13" s="3">
         <f>($AA13-AJ13-AM13)*AO5%</f>
-        <v>3.1232879999999996</v>
+        <v>0</v>
       </c>
       <c r="AS13" s="3">
         <f t="shared" si="1"/>
-        <v>11.036452000000001</v>
+        <v>0</v>
       </c>
       <c r="AU13" s="3">
         <f t="shared" si="2"/>
-        <v>239.10354799999999</v>
+        <v>0</v>
       </c>
       <c r="BA13" s="3">
         <f t="shared" si="3"/>
-        <v>31.08242576</v>
+        <v>0</v>
       </c>
       <c r="BB13" s="3">
         <f t="shared" si="4"/>
-        <v>270.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D14" s="7"/>
       <c r="AA14" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>250.14</v>
       </c>
       <c r="AE14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.776554</v>
       </c>
       <c r="AG14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.8766099999999999</v>
       </c>
       <c r="AJ14" s="3">
         <f>$R6*AI6</f>
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AM14" s="3">
         <f>$R6*AL6</f>
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AP14" s="3">
         <f>($AA14-AJ14-AM14)*AO6%</f>
-        <v>0</v>
+        <v>3.1232879999999996</v>
       </c>
       <c r="AS14" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>11.036452000000001</v>
       </c>
       <c r="AU14" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>239.10354799999999</v>
       </c>
       <c r="BA14" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31.08242576</v>
       </c>
       <c r="BB14" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>270.19</v>
       </c>
     </row>
     <row r="15" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[Vikas]Updated transactions in the Finance and Production modules, along with their corresponding Excel files, and made modifications to a few classes
</commit_message>
<xml_diff>
--- a/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
+++ b/src/main/resources/menuItems/Sales/Transactions/480464 - Sales Return with Invoice Reference-AC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\Wings-Automation\src\main\resources\menuItems\Sales\Transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6DAC46-8B8B-48F1-A9B4-AF5F47CDD76F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E339B17E-2C18-497D-8B3B-030FBE144B68}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="938" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5950,7 +5950,7 @@
         <v>192</v>
       </c>
       <c r="J5" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="K5" t="s">
         <v>194</v>
@@ -5968,40 +5968,40 @@
         <v>142</v>
       </c>
       <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
         <v>1</v>
       </c>
-      <c r="Q5">
+      <c r="U5">
         <v>1</v>
       </c>
-      <c r="R5">
+      <c r="V5">
         <v>1</v>
       </c>
-      <c r="S5">
+      <c r="W5">
         <v>1</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
       </c>
       <c r="X5">
         <v>500.14</v>
       </c>
       <c r="Y5">
-        <v>500.14</v>
+        <v>0</v>
       </c>
       <c r="Z5">
         <v>250.14</v>
       </c>
       <c r="AA5">
-        <v>250.14</v>
+        <v>0</v>
       </c>
       <c r="AB5" s="5">
         <v>0</v>
@@ -6013,13 +6013,13 @@
         <v>1.1100000000000001</v>
       </c>
       <c r="AE5">
-        <v>2.78</v>
+        <v>0</v>
       </c>
       <c r="AF5">
-        <v>1.1499999999999999</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="AG5">
-        <v>2.88</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="s">
         <v>195</v>
@@ -6028,7 +6028,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ5">
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="s">
         <v>195</v>
@@ -6037,7 +6037,7 @@
         <v>1.21</v>
       </c>
       <c r="AM5">
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AN5" t="s">
         <v>196</v>
@@ -6046,7 +6046,7 @@
         <v>1.26</v>
       </c>
       <c r="AP5">
-        <v>3.12</v>
+        <v>0</v>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -6061,31 +6061,31 @@
         <v>146</v>
       </c>
       <c r="AU5">
-        <v>239.1</v>
+        <v>0</v>
       </c>
       <c r="AV5">
         <v>12</v>
       </c>
       <c r="AW5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AX5">
-        <v>14.35</v>
+        <v>0</v>
       </c>
       <c r="AY5">
         <v>0</v>
       </c>
       <c r="AZ5">
-        <v>2.39</v>
+        <v>0</v>
       </c>
       <c r="BA5">
-        <v>31.09</v>
+        <v>0</v>
       </c>
       <c r="BB5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BC5">
-        <v>270.19</v>
+        <v>0</v>
       </c>
       <c r="BD5" t="s">
         <v>197</v>
@@ -6100,46 +6100,46 @@
         <v>200</v>
       </c>
       <c r="BH5" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="BI5" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="BJ5" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="BK5" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="BL5" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="BM5" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="BN5">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="BO5">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="BP5">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="BQ5">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="BR5">
-        <v>1.58</v>
+        <v>1.59</v>
       </c>
       <c r="BS5" s="1">
-        <v>45859</v>
+        <v>45862</v>
       </c>
       <c r="BT5" s="1">
-        <v>45860</v>
+        <v>45863</v>
       </c>
       <c r="BU5" s="1">
-        <v>45861</v>
+        <v>45864</v>
       </c>
       <c r="BV5" s="6">
         <v>1</v>
@@ -6180,7 +6180,7 @@
         <v>192</v>
       </c>
       <c r="J6" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="K6" t="s">
         <v>194</v>
@@ -6198,40 +6198,40 @@
         <v>142</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6">
         <v>500.14</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <v>500.14</v>
       </c>
       <c r="Z6">
         <v>250.14</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <v>250.14</v>
       </c>
       <c r="AB6" s="5">
         <v>0</v>
@@ -6243,13 +6243,13 @@
         <v>1.1100000000000001</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <v>2.78</v>
       </c>
       <c r="AF6">
-        <v>1.1599999999999999</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <v>2.88</v>
       </c>
       <c r="AH6" t="s">
         <v>195</v>
@@ -6258,7 +6258,7 @@
         <v>1.05</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AK6" t="s">
         <v>195</v>
@@ -6267,7 +6267,7 @@
         <v>1.21</v>
       </c>
       <c r="AM6">
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AN6" t="s">
         <v>196</v>
@@ -6276,7 +6276,7 @@
         <v>1.26</v>
       </c>
       <c r="AP6">
-        <v>0</v>
+        <v>3.12</v>
       </c>
       <c r="AQ6">
         <v>0</v>
@@ -6291,31 +6291,31 @@
         <v>146</v>
       </c>
       <c r="AU6">
-        <v>0</v>
+        <v>239.1</v>
       </c>
       <c r="AV6">
         <v>12</v>
       </c>
       <c r="AW6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AX6">
-        <v>0</v>
+        <v>14.35</v>
       </c>
       <c r="AY6">
         <v>0</v>
       </c>
       <c r="AZ6">
-        <v>0</v>
+        <v>2.39</v>
       </c>
       <c r="BA6">
-        <v>0</v>
+        <v>31.09</v>
       </c>
       <c r="BB6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BC6">
-        <v>0</v>
+        <v>270.19</v>
       </c>
       <c r="BD6" t="s">
         <v>197</v>
@@ -6330,46 +6330,46 @@
         <v>200</v>
       </c>
       <c r="BH6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="BI6" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="BJ6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="BK6" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="BL6" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="BM6" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="BN6">
-        <v>1.33</v>
+        <v>1.32</v>
       </c>
       <c r="BO6">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
       <c r="BP6">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="BQ6">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="BR6">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
       <c r="BS6" s="1">
-        <v>45862</v>
+        <v>45859</v>
       </c>
       <c r="BT6" s="1">
-        <v>45863</v>
+        <v>45860</v>
       </c>
       <c r="BU6" s="1">
-        <v>45864</v>
+        <v>45861</v>
       </c>
       <c r="BV6" s="6">
         <v>1</v>
@@ -6747,86 +6747,86 @@
       <c r="D13" s="7"/>
       <c r="AA13" s="3">
         <f t="shared" si="0"/>
-        <v>250.14</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="3">
         <f t="shared" si="5"/>
-        <v>2.776554</v>
+        <v>0</v>
       </c>
       <c r="AG13" s="3">
         <f t="shared" si="5"/>
-        <v>2.8766099999999999</v>
+        <v>0</v>
       </c>
       <c r="AJ13" s="3">
         <f>$R5*AI5</f>
-        <v>1.05</v>
+        <v>0</v>
       </c>
       <c r="AM13" s="3">
         <f>$R5*AL5</f>
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="AP13" s="3">
         <f>($AA13-AJ13-AM13)*AO5%</f>
-        <v>3.1232879999999996</v>
+        <v>0</v>
       </c>
       <c r="AS13" s="3">
         <f t="shared" si="1"/>
-        <v>11.036452000000001</v>
+        <v>0</v>
       </c>
       <c r="AU13" s="3">
         <f t="shared" si="2"/>
-        <v>239.10354799999999</v>
+        <v>0</v>
       </c>
       <c r="BA13" s="3">
         <f t="shared" si="3"/>
-        <v>31.08242576</v>
+        <v>0</v>
       </c>
       <c r="BB13" s="3">
         <f t="shared" si="4"/>
-        <v>270.19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D14" s="7"/>
       <c r="AA14" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>250.14</v>
       </c>
       <c r="AE14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.776554</v>
       </c>
       <c r="AG14" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.8766099999999999</v>
       </c>
       <c r="AJ14" s="3">
         <f>$R6*AI6</f>
-        <v>0</v>
+        <v>1.05</v>
       </c>
       <c r="AM14" s="3">
         <f>$R6*AL6</f>
-        <v>0</v>
+        <v>1.21</v>
       </c>
       <c r="AP14" s="3">
         <f>($AA14-AJ14-AM14)*AO6%</f>
-        <v>0</v>
+        <v>3.1232879999999996</v>
       </c>
       <c r="AS14" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>11.036452000000001</v>
       </c>
       <c r="AU14" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>239.10354799999999</v>
       </c>
       <c r="BA14" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31.08242576</v>
       </c>
       <c r="BB14" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>270.19</v>
       </c>
     </row>
     <row r="15" spans="1:76" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>